<commit_message>
Renforcer la reproduction et clarifier les résultats après audit
</commit_message>
<xml_diff>
--- a/results/resultats.xlsx
+++ b/results/resultats.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Résultats" sheetId="1" r:id="Rc4327b21a638493c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prévisions" sheetId="2" r:id="R90cd4d72a1344427"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemple" sheetId="3" r:id="Re340188117984702"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Résultats" sheetId="1" r:id="Rba56c62a21274594"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prévisions" sheetId="2" r:id="R409aca854db14783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemple" sheetId="3" r:id="Rccb6fb1413244521"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -699,7 +699,7 @@
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
       <x:c r="A9" s="19" t="str">
-        <x:v>Australia</x:v>
+        <x:v>Australie</x:v>
       </x:c>
       <x:c r="B9" s="13" t="n">
         <x:v>36</x:v>
@@ -717,7 +717,7 @@
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
       <x:c r="A10" s="16" t="str">
-        <x:v>Belgium</x:v>
+        <x:v>Belgique</x:v>
       </x:c>
       <x:c r="B10" s="10" t="n">
         <x:v>36</x:v>
@@ -735,7 +735,7 @@
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
       <x:c r="A11" s="19" t="str">
-        <x:v>Switzerland</x:v>
+        <x:v>Suisse</x:v>
       </x:c>
       <x:c r="B11" s="13" t="n">
         <x:v>36</x:v>
@@ -753,7 +753,7 @@
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
       <x:c r="A12" s="16" t="str">
-        <x:v>Germany</x:v>
+        <x:v>Allemagne</x:v>
       </x:c>
       <x:c r="B12" s="10" t="n">
         <x:v>36</x:v>
@@ -771,7 +771,7 @@
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
       <x:c r="A13" s="19" t="str">
-        <x:v>Denmark</x:v>
+        <x:v>Danemark</x:v>
       </x:c>
       <x:c r="B13" s="13" t="n">
         <x:v>36</x:v>
@@ -789,7 +789,7 @@
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
       <x:c r="A14" s="16" t="str">
-        <x:v>Spain</x:v>
+        <x:v>Espagne</x:v>
       </x:c>
       <x:c r="B14" s="10" t="n">
         <x:v>36</x:v>
@@ -807,7 +807,7 @@
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
       <x:c r="A15" s="19" t="str">
-        <x:v>Finland</x:v>
+        <x:v>Finlande</x:v>
       </x:c>
       <x:c r="B15" s="13" t="n">
         <x:v>36</x:v>
@@ -843,7 +843,7 @@
     </x:row>
     <x:row r="17" ht="22" customHeight="1">
       <x:c r="A17" s="19" t="str">
-        <x:v>UK</x:v>
+        <x:v>Royaume-Uni</x:v>
       </x:c>
       <x:c r="B17" s="13" t="n">
         <x:v>36</x:v>
@@ -861,7 +861,7 @@
     </x:row>
     <x:row r="18" ht="22" customHeight="1">
       <x:c r="A18" s="16" t="str">
-        <x:v>Italy</x:v>
+        <x:v>Italie</x:v>
       </x:c>
       <x:c r="B18" s="10" t="n">
         <x:v>36</x:v>
@@ -879,7 +879,7 @@
     </x:row>
     <x:row r="19" ht="22" customHeight="1">
       <x:c r="A19" s="19" t="str">
-        <x:v>Japan</x:v>
+        <x:v>Japon</x:v>
       </x:c>
       <x:c r="B19" s="13" t="n">
         <x:v>36</x:v>
@@ -897,7 +897,7 @@
     </x:row>
     <x:row r="20" ht="22" customHeight="1">
       <x:c r="A20" s="16" t="str">
-        <x:v>Netherlands</x:v>
+        <x:v>Pays-Bas</x:v>
       </x:c>
       <x:c r="B20" s="10" t="n">
         <x:v>36</x:v>
@@ -915,7 +915,7 @@
     </x:row>
     <x:row r="21" ht="22" customHeight="1">
       <x:c r="A21" s="19" t="str">
-        <x:v>Norway</x:v>
+        <x:v>Norvège</x:v>
       </x:c>
       <x:c r="B21" s="13" t="n">
         <x:v>36</x:v>
@@ -951,7 +951,7 @@
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
       <x:c r="A23" s="19" t="str">
-        <x:v>Sweden</x:v>
+        <x:v>Suède</x:v>
       </x:c>
       <x:c r="B23" s="13" t="n">
         <x:v>36</x:v>
@@ -969,7 +969,7 @@
     </x:row>
     <x:row r="24" ht="22" customHeight="1">
       <x:c r="A24" s="16" t="str">
-        <x:v>USA</x:v>
+        <x:v>États-Unis</x:v>
       </x:c>
       <x:c r="B24" s="10" t="n">
         <x:v>36</x:v>

</xml_diff>